<commit_message>
feat(weightedIFCCalculation): small fixes and calculating new deciles match
</commit_message>
<xml_diff>
--- a/IFC_Italy_2018_reference_points.xlsx
+++ b/IFC_Italy_2018_reference_points.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t xml:space="preserve">reference_area</t>
   </si>
@@ -26,7 +26,7 @@
     <t xml:space="preserve">I2_ref</t>
   </si>
   <si>
-    <t xml:space="preserve">I3_ref</t>
+    <t xml:space="preserve">I3_ref_approx</t>
   </si>
   <si>
     <t xml:space="preserve">I4_ref</t>
@@ -35,7 +35,7 @@
     <t xml:space="preserve">I5_ref</t>
   </si>
   <si>
-    <t xml:space="preserve">I6_ref_approx</t>
+    <t xml:space="preserve">I6_ref</t>
   </si>
   <si>
     <t xml:space="preserve">I7_ref</t>
@@ -50,28 +50,43 @@
     <t xml:space="preserve">I10_ref</t>
   </si>
   <si>
-    <t xml:space="preserve">I11_ref_exact</t>
+    <t xml:space="preserve">I11_ref</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I11_ref_raw_density_info_only</t>
   </si>
   <si>
     <t xml:space="preserve">I12_ref_rough_employment_weighted_ventile</t>
   </si>
   <si>
+    <t xml:space="preserve">note_order</t>
+  </si>
+  <si>
     <t xml:space="preserve">note_I3</t>
   </si>
   <si>
     <t xml:space="preserve">note_I6</t>
   </si>
   <si>
+    <t xml:space="preserve">note_I11</t>
+  </si>
+  <si>
     <t xml:space="preserve">note_I12</t>
   </si>
   <si>
     <t xml:space="preserve">Italy</t>
   </si>
   <si>
+    <t xml:space="preserve">Workbook order: I1 cars, I2 waste, I3 protected, I4 landslides, I5 soil, I6 accessibility, I7 dependency, I8 education, I9 employment, I10 migration, I11 LU ventile, I12 low-productivity ventile.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approximation: area-weighted municipal protected-area value; official numerator is GIS protected-area overlay and may use different surfaces.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Simple municipal mean; accessibility has no natural additive denominator.</t>
   </si>
   <si>
-    <t xml:space="preserve">Approximation: area-weighted municipal value; official numerator is GIS protected-area overlay and may use different surfaces.</t>
+    <t xml:space="preserve">Municipal Ind11 is a ventile/class (1-20). The script computes Italy raw LU density from totals, then converts it to the corresponding 2018 municipal ventile class; raw density is reported only as info.</t>
   </si>
   <si>
     <t xml:space="preserve">Rough approximation: employment-weighted mean of municipal ventiles/classes; exact raw value needs Frame-SBS Territorial low-productivity numerator.</t>
@@ -407,19 +422,22 @@
     <col min="2" max="2" width="14.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="11.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="11.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="13.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="11.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="11.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="13.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
     <col min="11" max="11" width="11.71" hidden="0" customWidth="1"/>
     <col min="12" max="12" width="11.71" hidden="0" customWidth="1"/>
-    <col min="13" max="13" width="13.71" hidden="0" customWidth="1"/>
-    <col min="14" max="14" width="41.71" hidden="0" customWidth="1"/>
-    <col min="15" max="15" width="73.71" hidden="0" customWidth="1"/>
-    <col min="16" max="16" width="126.71" hidden="0" customWidth="1"/>
-    <col min="17" max="17" width="148.71" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="7.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="29.71" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="41.71" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="195.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="141.71" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="73.71" hidden="0" customWidth="1"/>
+    <col min="19" max="19" width="202.71" hidden="0" customWidth="1"/>
+    <col min="20" max="20" width="148.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -474,58 +492,76 @@
       <c r="Q1" t="s">
         <v>16</v>
       </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B2" t="n">
         <v>2018</v>
       </c>
       <c r="C2" t="n">
-        <v>5.44001689681807</v>
+        <v>22.9317143244857</v>
       </c>
       <c r="D2" t="n">
-        <v>27.1929359920132</v>
+        <v>208.671548586661</v>
       </c>
       <c r="E2" t="n">
-        <v>175.576320360041</v>
+        <v>21.6154297449356</v>
       </c>
       <c r="F2" t="n">
-        <v>13.5395299741921</v>
+        <v>8.41676532884506</v>
       </c>
       <c r="G2" t="n">
-        <v>5.00915267457308</v>
+        <v>7.0500662072612</v>
       </c>
       <c r="H2" t="n">
-        <v>7.0500662072612</v>
+        <v>31.0973694219067</v>
       </c>
       <c r="I2" t="n">
-        <v>16.9110567905459</v>
+        <v>69.080945159912</v>
       </c>
       <c r="J2" t="n">
-        <v>69.0992288802015</v>
+        <v>36.7306426317974</v>
       </c>
       <c r="K2" t="n">
-        <v>36.7805995793175</v>
+        <v>63.068621550296</v>
       </c>
       <c r="L2" t="n">
-        <v>63.0413375674731</v>
+        <v>13.6517891888504</v>
       </c>
       <c r="M2" t="n">
+        <v>16</v>
+      </c>
+      <c r="N2" t="n">
         <v>79.5972747517884</v>
       </c>
-      <c r="N2" t="n">
-        <v>15.7360930035439</v>
-      </c>
-      <c r="O2" t="s">
-        <v>18</v>
+      <c r="O2" t="n">
+        <v>8.28234865437325</v>
       </c>
       <c r="P2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="Q2" t="s">
-        <v>20</v>
+        <v>22</v>
+      </c>
+      <c r="R2" t="s">
+        <v>23</v>
+      </c>
+      <c r="S2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T2" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>